<commit_message>
📊 Horarios actualizados Línea 141 - 3256
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-07.xlsx
+++ b/data/horarios-141-2026-06-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:58:28</t>
+          <t>Última actualización: 05:22:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:58:28</t>
+          <t>05:22:07</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:01</t>
+          <t>05:24</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>63</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01:58:28</t>
+          <t>05:22:07</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,23 +523,273 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>01:58:28</t>
+          <t>05:22:07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>110</v>
+        <v>25</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>05:22:07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>39</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>05:22:07</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06:09</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>47</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>05:22:07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06:13</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>51</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>05:22:07</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>68</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>05:22:07</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06:36</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>74</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>05:22:07</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>77</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>05:22:07</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>79</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>05:22:07</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>79</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>05:22:07</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06:59</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>97</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>05:22:07</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07:03</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>101</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -556,7 +806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,14 +819,91 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:58:28</t>
+          <t>Última actualización: 05:22:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>05:22:07</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06:13</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>51</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>05:22:07</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:03</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>101</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -604,7 +931,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:58:28</t>
+          <t>Última actualización: 05:22:07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3257
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-07.xlsx
+++ b/data/horarios-141-2026-06-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:22:07</t>
+          <t>Última actualización: 07:38:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:22:07</t>
+          <t>07:38:59</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:24</t>
+          <t>07:39</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:22:07</t>
+          <t>07:38:59</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>07:43</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:22:07</t>
+          <t>07:38:59</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,12 +548,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:22:07</t>
+          <t>07:38:59</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:22:07</t>
+          <t>07:38:59</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>08:05</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:22:07</t>
+          <t>07:38:59</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:13</t>
+          <t>08:18</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,12 +623,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:22:07</t>
+          <t>07:38:59</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:22:07</t>
+          <t>07:38:59</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:36</t>
+          <t>08:25</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:22:07</t>
+          <t>07:38:59</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:22:07</t>
+          <t>07:38:59</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:22:07</t>
+          <t>07:38:59</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>09:03</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:22:07</t>
+          <t>07:38:59</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,23 +773,148 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:22:07</t>
+          <t>07:38:59</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:03</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>07:38:59</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>98</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>07:38:59</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>98</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>07:38:59</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>09:23</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>105</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>07:38:59</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>09:33</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>115</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>07:38:59</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>116</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -806,7 +931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -819,14 +944,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:22:07</t>
+          <t>Última actualización: 07:38:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -860,12 +985,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:22:07</t>
+          <t>07:38:59</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06:13</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -874,7 +999,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>51</v>
+        <v>13</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -885,23 +1010,73 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:22:07</t>
+          <t>07:38:59</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07:03</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>66</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>07:38:59</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>66</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:38:59</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>101</v>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="D9" t="n">
+        <v>88</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -918,7 +1093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -931,14 +1106,116 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:22:07</t>
+          <t>Última actualización: 07:38:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>07:38:59</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>07:38:59</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>08:37</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>59</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>07:38:59</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>09:02</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>84</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3258
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-07.xlsx
+++ b/data/horarios-141-2026-06-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:38:59</t>
+          <t>Última actualización: 09:10:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>07:38:59</t>
+          <t>09:10:53</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>98</v>
+        <v>6</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07:38:59</t>
+          <t>09:10:53</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -837,7 +837,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>98</v>
+        <v>6</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:38:59</t>
+          <t>09:10:53</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -862,7 +862,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>105</v>
+        <v>13</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07:38:59</t>
+          <t>09:10:53</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,13 +908,413 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>24</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>07:38:59</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D24" t="n">
         <v>116</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>25</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>09:36</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>26</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>34</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>41</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>44</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10:03</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>53</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>65</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>74</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>84</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>93</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>10:48</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>98</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>105</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>106</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>114</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>11:07</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>117</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -931,7 +1331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -944,14 +1344,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:38:59</t>
+          <t>Última actualización: 09:10:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -1077,6 +1477,31 @@
         <v>88</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>44</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1093,7 +1518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1106,14 +1531,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:38:59</t>
+          <t>Última actualización: 09:10:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1216,6 +1641,106 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>17</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>10:17</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>67</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10:29</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>79</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>09:10:53</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>92</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3259
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-07.xlsx
+++ b/data/horarios-141-2026-06-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:10:53</t>
+          <t>Última actualización: 11:20:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 52</t>
         </is>
       </c>
     </row>
@@ -1315,6 +1315,456 @@
         <v>117</v>
       </c>
       <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>11:24</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>4</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>14</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>11:36</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>16</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>11:41</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>21</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>24</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>34</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>35</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>44</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>55</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>12:24</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>64</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>73</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>74</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>74</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>84</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>86</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>94</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>104</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>115</v>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1331,7 +1781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1344,14 +1794,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:10:53</t>
+          <t>Última actualización: 11:20:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1502,6 +1952,81 @@
         <v>44</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>14</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>24</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>94</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1518,7 +2043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1531,14 +2056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:10:53</t>
+          <t>Última actualización: 11:20:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1741,6 +2266,31 @@
       <c r="E12" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>11:20:43</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3260
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-07.xlsx
+++ b/data/horarios-141-2026-06-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:20:43</t>
+          <t>Última actualización: 12:48:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 52</t>
+          <t>Total filas: 69</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>11:20:43</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>104</v>
+        <v>7</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1753,18 +1753,443 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>104</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>17</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
           <t>13:15</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D57" t="n">
-        <v>115</v>
-      </c>
-      <c r="E57" t="inlineStr">
+      <c r="D59" t="n">
+        <v>27</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>34</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>36</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>44</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>57</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>67</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>68</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>76</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>83</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>86</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>86</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>89</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>97</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>103</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>107</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>116</v>
+      </c>
+      <c r="E74" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1781,7 +2206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1794,14 +2219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:20:43</t>
+          <t>Última actualización: 12:48:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -2027,6 +2452,81 @@
         <v>94</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>7</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>44</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>107</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2043,7 +2543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2056,14 +2556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:20:43</t>
+          <t>Última actualización: 12:48:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -2289,6 +2789,81 @@
         <v>3</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>35</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>62</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>115</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3261
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-07.xlsx
+++ b/data/horarios-141-2026-06-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:48:06</t>
+          <t>Última actualización: 13:58:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 69</t>
+          <t>Total filas: 82</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1973,21 +1973,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:58:39</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>13:58</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:58:39</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>83</v>
+        <v>6</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:58:39</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>86</v>
+        <v>13</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:58:39</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>86</v>
+        <v>16</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:58:39</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:58:39</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>97</v>
+        <v>18</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2128,16 +2128,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>103</v>
+        <v>89</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,21 +2148,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:58:39</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>107</v>
+        <v>26</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2178,18 +2178,343 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>97</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>33</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>36</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>107</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
           <t>14:44</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C78" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D74" t="n">
-        <v>116</v>
-      </c>
-      <c r="E74" t="inlineStr">
+      <c r="D78" t="n">
+        <v>46</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>56</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>14:58</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>60</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>66</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>77</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>86</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>96</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>106</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>117</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>118</v>
+      </c>
+      <c r="E87" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2206,7 +2531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2219,14 +2544,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:48:06</t>
+          <t>Última actualización: 13:58:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2510,23 +2835,123 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>36</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>12:48:06</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>14:35</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D17" t="n">
         <v>107</v>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>56</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>66</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>96</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2543,7 +2968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2556,14 +2981,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:48:06</t>
+          <t>Última actualización: 13:58:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -2847,25 +3272,75 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>14:42</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>44</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>12:48:06</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>14:43</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D17" t="n">
         <v>115</v>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>15:22</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>84</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3262
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-07.xlsx
+++ b/data/horarios-141-2026-06-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E87"/>
+  <dimension ref="A1:E100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:58:39</t>
+          <t>Última actualización: 15:01:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 82</t>
+          <t>Total filas: 95</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:01:43</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>15:02</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>66</v>
+        <v>1</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,21 +2373,21 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:01:43</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:03</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>77</v>
+        <v>2</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:01:43</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>86</v>
+        <v>3</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:01:43</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>96</v>
+        <v>14</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:01:43</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>106</v>
+        <v>23</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:01:43</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>117</v>
+        <v>33</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,23 +2498,348 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
+          <t>15:01:43</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>40</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>15:01:43</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>43</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>15:01:43</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>15:53</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>52</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>15:01:43</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>54</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
           <t>13:58:39</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B91" t="inlineStr">
         <is>
           <t>15:56</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C91" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D87" t="n">
+      <c r="D91" t="n">
         <v>118</v>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>15:01:43</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>63</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>15:01:43</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>73</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>15:01:43</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>74</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>15:01:43</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>83</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>15:01:43</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>84</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>15:01:43</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>93</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>15:01:43</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>94</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>15:01:43</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>103</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>15:01:43</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>114</v>
+      </c>
+      <c r="E100" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2544,7 +2869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:58:39</t>
+          <t>Última actualización: 15:01:43</t>
         </is>
       </c>
     </row>
@@ -2910,7 +3235,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:01:43</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2924,7 +3249,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>66</v>
+        <v>3</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -2935,7 +3260,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:01:43</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2949,7 +3274,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>96</v>
+        <v>33</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2968,7 +3293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2981,14 +3306,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:58:39</t>
+          <t>Última actualización: 15:01:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -3341,6 +3666,31 @@
       <c r="E18" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>15:01:43</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>16:02</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>61</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3263
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-07.xlsx
+++ b/data/horarios-141-2026-06-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E100"/>
+  <dimension ref="A1:E115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:01:43</t>
+          <t>Última actualización: 16:43:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 95</t>
+          <t>Total filas: 110</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>09:10:53</t>
+          <t>07:38:59</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,11 +908,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>07:38:59</t>
+          <t>09:10:53</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -933,11 +933,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>15:01:43</t>
+          <t>16:43:28</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2812,7 +2812,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>103</v>
+        <v>1</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,23 +2823,398 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>15:01:43</t>
+          <t>16:43:28</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>8</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
           <t>16:55</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
+      <c r="C101" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D100" t="n">
-        <v>114</v>
-      </c>
-      <c r="E100" t="inlineStr">
+      <c r="D101" t="n">
+        <v>12</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>21</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>32</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>41</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>17:26</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>43</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>52</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>53</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>55</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>61</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>72</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>18:04</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>81</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>92</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>97</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>101</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>111</v>
+      </c>
+      <c r="E115" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2856,7 +3231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2869,14 +3244,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:01:43</t>
+          <t>Última actualización: 16:43:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -3277,6 +3652,106 @@
         <v>33</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>32</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>61</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>72</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>92</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3293,7 +3768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3306,14 +3781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:01:43</t>
+          <t>Última actualización: 16:43:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -3689,6 +4164,31 @@
         <v>61</v>
       </c>
       <c r="E19" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>16:43:28</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>40</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3264
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-07.xlsx
+++ b/data/horarios-141-2026-06-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E115"/>
+  <dimension ref="A1:E130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:43:28</t>
+          <t>Última actualización: 17:51:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 110</t>
+          <t>Total filas: 125</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>16:43:28</t>
+          <t>17:51:36</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3087,7 +3087,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>72</v>
+        <v>4</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>16:43:28</t>
+          <t>17:51:36</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>18:04</t>
+          <t>18:01</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>81</v>
+        <v>10</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>16:43:28</t>
+          <t>17:51:36</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>92</v>
+        <v>13</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>16:43:28</t>
+          <t>17:51:36</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:14</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>97</v>
+        <v>23</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3178,16 +3178,16 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3203,18 +3203,393 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>97</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>18:21</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>30</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>33</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
           <t>18:34</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr">
+      <c r="C118" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D115" t="n">
-        <v>111</v>
-      </c>
-      <c r="E115" t="inlineStr">
+      <c r="D118" t="n">
+        <v>43</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>45</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>53</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>63</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>69</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>73</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>19:12</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>81</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>85</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>85</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>93</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>93</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>118</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>119</v>
+      </c>
+      <c r="E130" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3231,7 +3606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3244,14 +3619,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:43:28</t>
+          <t>Última actualización: 17:51:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -3710,7 +4085,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>16:43:28</t>
+          <t>17:51:36</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3724,7 +4099,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>72</v>
+        <v>4</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -3735,23 +4110,98 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>18:14</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>23</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>16:43:28</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>18:15</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D25" t="n">
         <v>92</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>69</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>93</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3768,7 +4218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3781,14 +4231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:43:28</t>
+          <t>Última actualización: 17:51:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -4189,6 +4639,81 @@
         <v>40</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>53</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>84</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>17:51:36</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>19:46</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>115</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3265
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-07.xlsx
+++ b/data/horarios-141-2026-06-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E130"/>
+  <dimension ref="A1:E141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:51:36</t>
+          <t>Última actualización: 18:56:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 125</t>
+          <t>Total filas: 136</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -833,7 +833,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07:38:59</t>
+          <t>09:10:53</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,11 +908,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>09:10:53</t>
+          <t>07:38:59</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -933,11 +933,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>17:51:36</t>
+          <t>18:56:35</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:56</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>17:51:36</t>
+          <t>18:56:35</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>18:57</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>73</v>
+        <v>1</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>17:51:36</t>
+          <t>18:56:35</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>81</v>
+        <v>4</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>17:51:36</t>
+          <t>18:56:35</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>85</v>
+        <v>8</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>17:51:36</t>
+          <t>18:56:35</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>85</v>
+        <v>15</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3503,16 +3503,16 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3528,16 +3528,16 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>17:51:36</t>
+          <t>18:56:35</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>118</v>
+        <v>20</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3578,18 +3578,293 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>93</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>18:56:35</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>28</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>18:56:35</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>29</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>18:56:35</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>53</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>18:56:35</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
           <t>19:50</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr">
+      <c r="C134" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D130" t="n">
-        <v>119</v>
-      </c>
-      <c r="E130" t="inlineStr">
+      <c r="D134" t="n">
+        <v>54</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>18:56:35</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>19:58</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>62</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>18:56:35</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>79</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>18:56:35</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>79</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>18:56:35</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>86</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>18:56:35</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>20:36</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>100</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>18:56:35</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>103</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>18:56:35</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>106</v>
+      </c>
+      <c r="E141" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3606,7 +3881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3619,14 +3894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:51:36</t>
+          <t>Última actualización: 18:56:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -4160,7 +4435,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>17:51:36</t>
+          <t>18:56:35</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4174,7 +4449,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4202,6 +4477,81 @@
         <v>93</v>
       </c>
       <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>18:56:35</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>29</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>18:56:35</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>79</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>18:56:35</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>103</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4218,7 +4568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4231,14 +4581,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:51:36</t>
+          <t>Última actualización: 18:56:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -4672,7 +5022,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>17:51:36</t>
+          <t>18:56:35</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4686,7 +5036,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>84</v>
+        <v>19</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -4697,7 +5047,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>17:51:36</t>
+          <t>18:56:35</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4711,9 +5061,34 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="E23" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>18:56:35</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>103</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3266
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-07.xlsx
+++ b/data/horarios-141-2026-06-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E141"/>
+  <dimension ref="A1:E152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:56:35</t>
+          <t>Última actualización: 19:55:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 136</t>
+          <t>Total filas: 147</t>
         </is>
       </c>
     </row>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>18:56:35</t>
+          <t>19:55:51</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>19:58</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3728,16 +3728,16 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:58</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>79</v>
+        <v>62</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>18:56:35</t>
+          <t>19:55:51</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>18:56:35</t>
+          <t>19:55:51</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>86</v>
+        <v>19</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3803,16 +3803,16 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>20:36</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>18:56:35</t>
+          <t>19:55:51</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>103</v>
+        <v>20</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3853,18 +3853,293 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>86</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>19:55:51</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>40</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>18:56:35</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>20:36</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>100</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>19:55:51</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>44</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>19:55:51</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>46</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>18:56:35</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
           <t>20:42</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr">
+      <c r="C146" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D141" t="n">
+      <c r="D146" t="n">
         <v>106</v>
       </c>
-      <c r="E141" t="inlineStr">
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>19:55:51</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>20:54</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>59</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>19:55:51</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>61</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>19:55:51</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>70</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>19:55:51</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>71</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>19:55:51</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>99</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>19:55:51</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>101</v>
+      </c>
+      <c r="E152" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3881,7 +4156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3894,14 +4169,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:56:35</t>
+          <t>Última actualización: 19:55:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -4510,12 +4785,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>18:56:35</t>
+          <t>19:55:51</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -4524,7 +4799,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>79</v>
+        <v>19</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -4540,18 +4815,43 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>79</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>19:55:51</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>20:39</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>103</v>
-      </c>
-      <c r="E30" t="inlineStr">
+      <c r="D31" t="n">
+        <v>44</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4568,7 +4868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4581,14 +4881,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:56:35</t>
+          <t>Última actualización: 19:55:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -5072,23 +5372,73 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>19:55:51</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>20:38</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>43</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>18:56:35</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>20:39</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D25" t="n">
         <v>103</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>19:55:51</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>21:31</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>96</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3267
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-06-07.xlsx
+++ b/data/horarios-141-2026-06-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E152"/>
+  <dimension ref="A1:E165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:55:51</t>
+          <t>Última actualización: 20:57:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 147</t>
+          <t>Total filas: 160</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>17:51:36</t>
+          <t>18:56:35</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>85</v>
+        <v>20</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>18:56:35</t>
+          <t>17:51:36</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>20</v>
+        <v>85</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>17:51:36</t>
+          <t>18:56:35</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>93</v>
+        <v>28</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>18:56:35</t>
+          <t>17:51:36</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>28</v>
+        <v>93</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>19:55:51</t>
+          <t>20:57:41</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>20:58</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>19:55:51</t>
+          <t>20:57:41</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>71</v>
+        <v>8</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4103,16 +4103,16 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>99</v>
+        <v>71</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,23 +4123,348 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
+          <t>20:57:41</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>21:07</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>10</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
           <t>19:55:51</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr">
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>99</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>20:57:41</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>38</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>19:55:51</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
         <is>
           <t>21:36</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr">
+      <c r="C155" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D152" t="n">
+      <c r="D155" t="n">
         <v>101</v>
       </c>
-      <c r="E152" t="inlineStr">
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>20:57:41</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>40</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>20:57:41</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>43</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>20:57:41</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>61</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>20:57:41</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>22:03</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>66</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>20:57:41</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>22:07</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>70</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>20:57:41</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>89</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>20:57:41</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>22:36</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>99</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>20:57:41</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>22:40</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>103</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>20:57:41</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>22:40</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>103</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>20:57:41</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>22:55</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>118</v>
+      </c>
+      <c r="E165" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4156,7 +4481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4169,14 +4494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:55:51</t>
+          <t>Última actualización: 20:57:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -4852,6 +5177,31 @@
         <v>44</v>
       </c>
       <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>20:57:41</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>22:36</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>99</v>
+      </c>
+      <c r="E32" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4868,7 +5218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4881,14 +5231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:55:51</t>
+          <t>Última actualización: 20:57:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -5441,6 +5791,56 @@
       <c r="E26" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>20:57:41</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>21:33</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>36</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>20:57:41</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>22:08</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>71</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>